<commit_message>
data(training): set sales pilot assessment rules
</commit_message>
<xml_diff>
--- a/29-employee-testing-service/question_bank_template.xlsx
+++ b/29-employee-testing-service/question_bank_template.xlsx
@@ -19,7 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Вопросы'!$A$1:$M$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Варианты'!$A$1:$F$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Назначение_по_должности'!$A$1:$D$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Программы'!$A$1:$K$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Программы'!$A$1:$L$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Источники'!$A$1:$F$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Справочники'!$A$1:$E$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Инструкция'!$A$1:$B$7</definedName>
@@ -201,20 +201,21 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Таблица4" displayName="Таблица4" ref="A1:K2" headerRowCount="1">
-  <autoFilter ref="A1:K2"/>
-  <tableColumns count="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Таблица4" displayName="Таблица4" ref="A1:L2" headerRowCount="1">
+  <autoFilter ref="A1:L2"/>
+  <tableColumns count="12">
     <tableColumn id="1" name="Код программы"/>
     <tableColumn id="2" name="Название"/>
-    <tableColumn id="3" name="Официальная должность"/>
+    <tableColumn id="3" name="Официальные должности"/>
     <tableColumn id="4" name="Темы"/>
     <tableColumn id="5" name="Число вопросов"/>
     <tableColumn id="6" name="Время, минут"/>
     <tableColumn id="7" name="Порог, %"/>
     <tableColumn id="8" name="Попыток"/>
-    <tableColumn id="9" name="Срок результата, месяцев"/>
-    <tableColumn id="10" name="Статус"/>
-    <tableColumn id="11" name="Версия"/>
+    <tableColumn id="9" name="Период попыток"/>
+    <tableColumn id="10" name="Срок действия результата"/>
+    <tableColumn id="11" name="Статус"/>
+    <tableColumn id="12" name="Версия"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1"/>
 </table>
@@ -777,7 +778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -791,6 +792,7 @@
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -806,7 +808,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Официальная должность</t>
+          <t>Официальные должности</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -836,15 +838,20 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Срок результата, месяцев</t>
+          <t>Период попыток</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>Срок действия результата</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>Статус</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Версия</t>
         </is>
@@ -852,7 +859,7 @@
     </row>
     <row r="2"/>
   </sheetData>
-  <autoFilter ref="A1:K2"/>
+  <autoFilter ref="A1:L2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>